<commit_message>
sEPARACAO DE INSS E DESATIVADOS EM JANELAS SEPARADAS
</commit_message>
<xml_diff>
--- a/atestados paulo.xlsx
+++ b/atestados paulo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Unicompo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Unicompo\Documents\03_PYTHON1\08 - RH_Grafico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{478DDBE4-CC08-401F-B454-B87C3A9EDE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{009340B5-2BF0-4012-9FC0-BF4EE930C384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5AFAA449-5FA3-4566-962D-330DB209F351}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Função do colaborador</t>
   </si>
@@ -46,10 +46,7 @@
     <t>Houve Afastamento Pelo INSS?</t>
   </si>
   <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>NÃO</t>
+    <t>Ativo/Desligado</t>
   </si>
 </sst>
 </file>
@@ -452,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E3101BB-735F-4AA0-9842-D41B282C068E}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="48" bestFit="1" customWidth="1"/>
@@ -461,9 +458,10 @@
     <col min="4" max="4" width="4.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -482,176 +480,162 @@
       <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
-      <c r="F14" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
-      <c r="F15" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
-      <c r="F16" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
-      <c r="F17" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
-      <c r="F18" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>